<commit_message>
Implemented parallel execution using ThreadLocal WebDriver
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>username</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>problem_user</t>
   </si>
 </sst>
 </file>
@@ -305,6 +308,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>